<commit_message>
Atualiza├º├úo autom├ítica 2026-01-06 10:06
</commit_message>
<xml_diff>
--- a/data/gasto por funcionario.xlsx
+++ b/data/gasto por funcionario.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="11_AD4D361C20488DEA4E38A03A0CDF58B65ADEDD81" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B33B1C5B-D2FD-48CE-905D-3970FE93C3DE}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="11_AD4D361C20488DEA4E38A03A0CDF58B65ADEDD81" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{572F84A9-2AA7-429D-A4E8-5EA710638802}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Plan1" sheetId="1" r:id="rId1"/>
+    <sheet name="2025" sheetId="1" r:id="rId1"/>
+    <sheet name="2026" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="3">
   <si>
     <t>COLABORADORES</t>
   </si>
@@ -523,4 +524,102 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA1572FF-D3CF-41CD-B32F-A6C0D8E3E0F1}">
+  <dimension ref="B1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="1">
+        <v>45658</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="1">
+        <v>45689</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="1">
+        <v>45717</v>
+      </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="1">
+        <v>45748</v>
+      </c>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="1">
+        <v>45778</v>
+      </c>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="1">
+        <v>45809</v>
+      </c>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="1">
+        <v>45839</v>
+      </c>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B9" s="1">
+        <v>45870</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B10" s="1">
+        <v>45901</v>
+      </c>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B11" s="1">
+        <v>45931</v>
+      </c>
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B12" s="1">
+        <v>45962</v>
+      </c>
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="1">
+        <v>45992</v>
+      </c>
+      <c r="C13" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-19 11:37
</commit_message>
<xml_diff>
--- a/data/gasto por funcionario.xlsx
+++ b/data/gasto por funcionario.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="11_AD4D361C20488DEA4E38A03A0CDF58B65ADEDD81" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{572F84A9-2AA7-429D-A4E8-5EA710638802}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="11_AD4D361C20488DEA4E38A03A0CDF58B65ADEDD81" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83CCB07F-F914-45C8-9BE6-882BF8F4C4A5}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2025" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -49,13 +49,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -85,11 +105,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -379,145 +405,145 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="7" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B2" s="1">
+      <c r="B2" s="4">
         <v>45658</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="5">
         <v>339463</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="6">
         <v>63</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B3" s="1">
+      <c r="B3" s="4">
         <v>45689</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="5">
         <v>339265</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="6">
         <v>63</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B4" s="1">
+      <c r="B4" s="4">
         <v>45717</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="5">
         <v>340561</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="6">
         <v>63</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B5" s="1">
+      <c r="B5" s="4">
         <v>45748</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="5">
         <v>342625</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="6">
         <v>63</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="1">
+      <c r="B6" s="4">
         <v>45778</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="5">
         <v>361588</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="6">
         <v>63</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B7" s="1">
+      <c r="B7" s="4">
         <v>45809</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="5">
         <v>357447</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="6">
         <v>63</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B8" s="1">
+      <c r="B8" s="4">
         <v>45839</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="5">
         <v>357752</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="6">
         <v>63</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B9" s="1">
+      <c r="B9" s="4">
         <v>45870</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="5">
         <v>357552</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="6">
         <v>63</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B10" s="1">
+      <c r="B10" s="4">
         <v>45901</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="5">
         <v>357656</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="6">
         <v>63</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B11" s="1">
+      <c r="B11" s="4">
         <v>45931</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="5">
         <v>357758</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="6">
         <v>63</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B12" s="1">
+      <c r="B12" s="4">
         <v>45962</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="5">
         <v>357462</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="6">
         <v>63</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B13" s="1">
+      <c r="B13" s="4">
         <v>45992</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="5">
         <v>357662</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="6">
         <v>63</v>
       </c>
     </row>

</xml_diff>